<commit_message>
A row of height 0 is hidden, as Excel takes it: SUBTOTAL 101-111 and AGGREGATE skip it, and on a filtered sheet SUBTOTAL 1-11 and the structure operations, in a book, a session's setLayout and the thread pool's outline; the round trip's book zero-sizes went through Excel again and its values now equal the engine's, its known difference gone
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test/excel/xlsx/roundtrip/zero-sizes.xlsx
+++ b/test/excel/xlsx/roundtrip/zero-sizes.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/user/Library/Containers/com.microsoft.Excel/Data/tmp/fxlsx-47250/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/user/Library/Containers/com.microsoft.Excel/Data/tmp/fxlsx-62206/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6EC3A2BD-47E7-5043-B85F-19B7A6059F03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{11AAE65F-61CB-E545-A0EB-8FF1F479C691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>